<commit_message>
energy-fuel-type: fix generation docs draft 1.0.0
</commit_message>
<xml_diff>
--- a/energy-fuel-type/energy-fuel-type.xlsx
+++ b/energy-fuel-type/energy-fuel-type.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scrocca\Desktop\cefriel-github\controlled-vocabularies\base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FF0BAE-D9D2-407C-BDED-F9DB6114E145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67FDE156-AA52-4D73-A272-688CF787A814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -126,106 +126,106 @@
     <t>Ed Ooms (NDW)</t>
   </si>
   <si>
+    <t>Zero-emission energy types</t>
+  </si>
+  <si>
+    <t>http://data.europa.eu/eli/reg/2023/1804/oj</t>
+  </si>
+  <si>
+    <t>Electricity AC</t>
+  </si>
+  <si>
+    <t>Electricity DC</t>
+  </si>
+  <si>
+    <t>Hydrogen</t>
+  </si>
+  <si>
+    <t>Ammonia</t>
+  </si>
+  <si>
+    <t>Renewable fuels</t>
+  </si>
+  <si>
+    <t>Biomass-fuel</t>
+  </si>
+  <si>
+    <t>Biofuel</t>
+  </si>
+  <si>
+    <t>Biogas</t>
+  </si>
+  <si>
+    <t>Renewable synthetic fuel</t>
+  </si>
+  <si>
+    <t>Renewable ammonia</t>
+  </si>
+  <si>
+    <t>Non‑renewable alternative and transitional fossil fuels</t>
+  </si>
+  <si>
+    <t>Compressed natural gas</t>
+  </si>
+  <si>
+    <t>Liquefied natural gas</t>
+  </si>
+  <si>
+    <t>Liquefied petroleum gas</t>
+  </si>
+  <si>
+    <t>Non-renewable synthetic fuel</t>
+  </si>
+  <si>
+    <t>Fossil fuels</t>
+  </si>
+  <si>
+    <t>Petrol</t>
+  </si>
+  <si>
+    <t>Diesel</t>
+  </si>
+  <si>
+    <t>Class URI</t>
+  </si>
+  <si>
+    <t>http://data.europa.eu/eli/ontology#LegalResource</t>
+  </si>
+  <si>
+    <t>PREFIX</t>
+  </si>
+  <si>
+    <t>eli</t>
+  </si>
+  <si>
+    <t>http://data.europa.eu/eli/ontology#</t>
+  </si>
+  <si>
+    <t>rdf:type</t>
+  </si>
+  <si>
+    <t>rdfs:label@en</t>
+  </si>
+  <si>
+    <t>rdfs:description@en</t>
+  </si>
+  <si>
+    <t>eli:LegalResource</t>
+  </si>
+  <si>
+    <t>Alternative Fuel Infrastructure Regulation (AFIR) - Regulation No 2023/1804</t>
+  </si>
+  <si>
+    <t>Regulation (EU) 2023/1804 of the European Parliament and of the Council of 13 September 2023 on the deployment of alternative fuels infrastructure, and repealing Directive 2014/94/EU</t>
+  </si>
+  <si>
+    <t>Draft Controlled Vocabulary</t>
+  </si>
+  <si>
+    <t>Energy Fuel Type</t>
+  </si>
+  <si>
     <t>1.0.0</t>
-  </si>
-  <si>
-    <t>Zero-emission energy types</t>
-  </si>
-  <si>
-    <t>http://data.europa.eu/eli/reg/2023/1804/oj</t>
-  </si>
-  <si>
-    <t>Electricity AC</t>
-  </si>
-  <si>
-    <t>Electricity DC</t>
-  </si>
-  <si>
-    <t>Hydrogen</t>
-  </si>
-  <si>
-    <t>Ammonia</t>
-  </si>
-  <si>
-    <t>Renewable fuels</t>
-  </si>
-  <si>
-    <t>Biomass-fuel</t>
-  </si>
-  <si>
-    <t>Biofuel</t>
-  </si>
-  <si>
-    <t>Biogas</t>
-  </si>
-  <si>
-    <t>Renewable synthetic fuel</t>
-  </si>
-  <si>
-    <t>Renewable ammonia</t>
-  </si>
-  <si>
-    <t>Non‑renewable alternative and transitional fossil fuels</t>
-  </si>
-  <si>
-    <t>Compressed natural gas</t>
-  </si>
-  <si>
-    <t>Liquefied natural gas</t>
-  </si>
-  <si>
-    <t>Liquefied petroleum gas</t>
-  </si>
-  <si>
-    <t>Non-renewable synthetic fuel</t>
-  </si>
-  <si>
-    <t>Fossil fuels</t>
-  </si>
-  <si>
-    <t>Petrol</t>
-  </si>
-  <si>
-    <t>Diesel</t>
-  </si>
-  <si>
-    <t>Class URI</t>
-  </si>
-  <si>
-    <t>http://data.europa.eu/eli/ontology#LegalResource</t>
-  </si>
-  <si>
-    <t>PREFIX</t>
-  </si>
-  <si>
-    <t>eli</t>
-  </si>
-  <si>
-    <t>http://data.europa.eu/eli/ontology#</t>
-  </si>
-  <si>
-    <t>rdf:type</t>
-  </si>
-  <si>
-    <t>rdfs:label@en</t>
-  </si>
-  <si>
-    <t>rdfs:description@en</t>
-  </si>
-  <si>
-    <t>eli:LegalResource</t>
-  </si>
-  <si>
-    <t>Alternative Fuel Infrastructure Regulation (AFIR) - Regulation No 2023/1804</t>
-  </si>
-  <si>
-    <t>Regulation (EU) 2023/1804 of the European Parliament and of the Council of 13 September 2023 on the deployment of alternative fuels infrastructure, and repealing Directive 2014/94/EU</t>
-  </si>
-  <si>
-    <t>Draft Controlled Vocabulary</t>
-  </si>
-  <si>
-    <t>[CANDIDATE RELEASE] Energy Fuel Type</t>
   </si>
 </sst>
 </file>
@@ -341,10 +341,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -661,7 +657,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -725,7 +721,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -756,7 +752,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -794,7 +790,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/zero-emission-energy-types</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="12"/>
@@ -805,7 +801,7 @@
       <c r="F19" s="10"/>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -814,7 +810,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/electricity-ac</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="12"/>
@@ -825,7 +821,7 @@
       </c>
       <c r="H20" s="1"/>
       <c r="I20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -834,7 +830,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/electricity-dc</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="12"/>
@@ -842,7 +838,7 @@
       <c r="F21" s="10"/>
       <c r="H21" s="1"/>
       <c r="I21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -851,7 +847,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/hydrogen</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="12"/>
@@ -862,7 +858,7 @@
       </c>
       <c r="H22" s="1"/>
       <c r="I22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -871,7 +867,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/ammonia</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="12"/>
@@ -882,7 +878,7 @@
       </c>
       <c r="H23" s="1"/>
       <c r="I23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -891,7 +887,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/renewable-fuels</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="12"/>
@@ -902,7 +898,7 @@
       <c r="F24" s="10"/>
       <c r="H24" s="1"/>
       <c r="I24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -911,7 +907,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/biomass-fuel</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="12"/>
@@ -922,7 +918,7 @@
       </c>
       <c r="H25" s="1"/>
       <c r="I25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -931,14 +927,14 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/biofuel</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F26" s="10" t="str">
         <f>A24</f>
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/renewable-fuels</v>
       </c>
       <c r="I26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -947,14 +943,14 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/biogas</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F27" s="10" t="str">
         <f>A24</f>
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/renewable-fuels</v>
       </c>
       <c r="I27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -963,14 +959,14 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/renewable-synthetic-fuel</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F28" s="10" t="str">
         <f>A24</f>
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/renewable-fuels</v>
       </c>
       <c r="I28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -979,14 +975,14 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/renewable-ammonia</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F29" s="10" t="str">
         <f>A24</f>
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/renewable-fuels</v>
       </c>
       <c r="I29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -995,7 +991,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/non‑renewable-alternative-and-transitional-fossil-fuels</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E30" s="1" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A31:A34)</f>
@@ -1003,7 +999,7 @@
       </c>
       <c r="F30" s="10"/>
       <c r="I30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1012,14 +1008,14 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/compressed-natural-gas</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F31" s="10" t="str">
         <f>A30</f>
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/non‑renewable-alternative-and-transitional-fossil-fuels</v>
       </c>
       <c r="I31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1028,14 +1024,14 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/liquefied-natural-gas</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F32" s="10" t="str">
         <f>A30</f>
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/non‑renewable-alternative-and-transitional-fossil-fuels</v>
       </c>
       <c r="I32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1044,14 +1040,14 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/liquefied-petroleum-gas</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F33" s="10" t="str">
         <f>A30</f>
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/non‑renewable-alternative-and-transitional-fossil-fuels</v>
       </c>
       <c r="I33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1060,14 +1056,14 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/non-renewable-synthetic-fuel</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F34" s="10" t="str">
         <f>A30</f>
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/non‑renewable-alternative-and-transitional-fossil-fuels</v>
       </c>
       <c r="I34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1076,7 +1072,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/fossil-fuels</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E35" s="1" t="str">
         <f>_xlfn.TEXTJOIN(", ",,A36:A37)</f>
@@ -1090,7 +1086,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/petrol</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F36" s="10" t="str">
         <f>A35</f>
@@ -1103,7 +1099,7 @@
         <v>https://w3id.org/mobilitydcat-ap/energy-fuel-type/diesel</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F37" s="10" t="str">
         <f>A35</f>
@@ -1148,22 +1144,22 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="C1" s="5"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
         <v>52</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1171,27 +1167,27 @@
         <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B7" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="D7" s="11" t="s">
         <v>59</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>